<commit_message>
Actualizar Excel clientes: tamañoEmpresa, correcciones idioma, pestaña análisis regenerada
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88153b17ae7a9f01/documentos/TRABAJOS AUTONOMOS/JURADA/j-busqueda clientes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="686" documentId="11_A9F854B1BC61342BED428D976AB7AEFF89D0661B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEB1D1AE-8907-5784-80C4-B6F8128DDC02}"/>
+  <xr:revisionPtr revIDLastSave="1347" documentId="11_A9F854B1BC61342BED428D976AB7AEFF89D0661B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2980377-10DC-42A0-BBAB-1369BD199A61}"/>
   <bookViews>
-    <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clientes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,6 @@
     <definedName name="DatosExternos_1" localSheetId="0">clientes!$A$1:$X$58</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -54,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3649" uniqueCount="2101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3712" uniqueCount="2100">
   <si>
     <t>fechaEmail</t>
   </si>
@@ -6112,12 +6111,6 @@
     <t>sudáfrica</t>
   </si>
   <si>
-    <t>ANÁLISIS DE FACTORES DE RESPUESTA</t>
-  </si>
-  <si>
-    <t>Actualizado: 19/02/2026</t>
-  </si>
-  <si>
     <t>HITOS CLAVE</t>
   </si>
   <si>
@@ -6127,33 +6120,15 @@
     <t>~29/01/2026: CV con 2 recomendaciones de clientes (1 de visados)</t>
   </si>
   <si>
-    <t>Análisis previo (nov 2025): email particular 46% vs genérico 36% respuesta</t>
-  </si>
-  <si>
-    <t>CLASIFICACIÓN DE RESPUESTAS USADA EN ESTE ANÁLISIS</t>
-  </si>
-  <si>
-    <t>POSITIVO REAL (interés comercial concreto):</t>
-  </si>
-  <si>
     <t>PT, PIDE PRES, PP, PPE, QG, R, R-C, TW</t>
   </si>
   <si>
-    <t>POSITIVO BLANDO (buena disposición sin acción):</t>
-  </si>
-  <si>
-    <t>POSITIVA, POSITIVO, PV, NP, AP, MP, MR, ME RECOMIENDA, ME REDIRIGE</t>
-  </si>
-  <si>
     <t>NEGATIVO:</t>
   </si>
   <si>
     <t>N, negativa, "ya tienen gente"</t>
   </si>
   <si>
-    <t>SIN EFECTO (email no llegó):</t>
-  </si>
-  <si>
     <t>SIN RESPUESTA:</t>
   </si>
   <si>
@@ -6193,18 +6168,12 @@
     <t>TIEMPO DE RESPUESTA</t>
   </si>
   <si>
-    <t>Media: 20 días | Mediana: 4 días</t>
-  </si>
-  <si>
     <t>DETALLE: RESPUESTAS POSITIVO REAL</t>
   </si>
   <si>
     <t>Empresa</t>
   </si>
   <si>
-    <t>Fecha email</t>
-  </si>
-  <si>
     <t>Email único</t>
   </si>
   <si>
@@ -6268,9 +6237,6 @@
     <t>FACTOR: PERSONALIZADO (col E): ¿mensaje personalizado?</t>
   </si>
   <si>
-    <t>medio</t>
-  </si>
-  <si>
     <t>FACTOR: IDIOMA (col M): ¿en inglés o español?</t>
   </si>
   <si>
@@ -6295,100 +6261,130 @@
     <t>FACTOR: REMINDER (col B): ¿se envió follow-up?</t>
   </si>
   <si>
-    <t>CONCLUSIONES</t>
-  </si>
-  <si>
-    <t>1. IDIOMA: DATO NO FIABLE — la columna M solo está rellenada en 90 de 271 filas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Los 3 PT (dan trabajo): 2 escritos en español (col M vacía), 1 en inglés.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   El análisis mostraba en&gt;es, pero es un espejismo por datos incompletos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   No se puede concluir nada sobre idioma hasta rellenar la columna M.</t>
-  </si>
-  <si>
-    <t>2. REGIÓN: España concentra los mejores resultados reales.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Los 3 clientes que han dado trabajo (PT) operan en España.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   5 de 7 Positivo Real con región conocida son de España.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   UK: 23% responde pero 0% Positivo Real (prefieren traductores locales).</t>
-  </si>
-  <si>
-    <t>3. REMINDERS: Los follow-up aumentan el Positivo Real (4.9% vs 2.2% sin reminder).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Insistir funciona para convertir interés latente en acción.</t>
-  </si>
-  <si>
-    <t>4. EMAIL PERSONAL vs GENÉRICO: Confirma análisis previo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Email personal: 26.7% positivo total vs genérico: 17.5%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Pero el % de Positivo Real es similar (~4%). La ventaja está en respuestas blandas.</t>
-  </si>
-  <si>
-    <t>5. PERSONALIZACIÓN: Los emails personalizados funcionan mejor (23.5% vs 15.8%).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Dado que casi todos son personalizados, este factor es difícil de aislar.</t>
-  </si>
-  <si>
-    <t>6. PERIODO TEMPORAL: Aún no se ve efecto claro de los cambios recientes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Antes ene-2026: 26.7% positivo (5.7% Real) — mejor tasa global.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Desde 29-ene (tarifa+recomendaciones): 20.4% (1.9% Real) — peor, pero...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   CAVEAT: los emails recientes no han tenido tiempo suficiente para generar respuestas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Este dato debe revisarse en 1-2 meses.</t>
-  </si>
-  <si>
-    <t>7. TASA GENERAL: 29% responde, 4% genera interés comercial real.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   De 271 contactadas, solo 11 mostraron interés real y 3 dieron trabajo.</t>
-  </si>
-  <si>
-    <t>CALIDAD DE DATOS — COLUMNAS CON MUCHOS VACÍOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Col M (idioma): solo 90/271 rellenadas (33%). Conclusiones no fiables.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Col N (adecuada): solo 25/271 rellenadas (9%). Muestra insuficiente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Col L (ubicación): 204/271 rellenadas (75%). Razonablemente fiable.</t>
-  </si>
-  <si>
-    <t>RECOMENDACIONES</t>
-  </si>
-  <si>
-    <t>• Priorizar empresas en España (o que operen en España)</t>
-  </si>
-  <si>
-    <t>• Seguir enviando reminders (aumentan conversión real)</t>
-  </si>
-  <si>
-    <t>• Rellenar col M (idioma) para poder evaluar ese factor con fiabilidad</t>
-  </si>
-  <si>
-    <t>• Revisar este análisis en abril 2026 para evaluar efecto de tarifa+recomendaciones</t>
+    <t>ANÁLISIS AMPLIADO DE FACTORES DE RESPUESTA</t>
+  </si>
+  <si>
+    <t>Actualizado: 21/02/2026</t>
+  </si>
+  <si>
+    <t>Incluye columnas Y (tipoPersonalización) y Z (tamañoEmpresa)</t>
+  </si>
+  <si>
+    <t>Feb 2026: análisis ampliado con datos de personalización y tamaño empresa</t>
+  </si>
+  <si>
+    <t>CLASIFICACIÓN DE RESPUESTAS</t>
+  </si>
+  <si>
+    <t>POSITIVO REAL:</t>
+  </si>
+  <si>
+    <t>POSITIVO BLANDO:</t>
+  </si>
+  <si>
+    <t>PV, NP, AP, MP, MR, ME RECOMIENDA, ME REDIRIGE</t>
+  </si>
+  <si>
+    <t>SIN EFECTO:</t>
+  </si>
+  <si>
+    <t>NE (email no llegó)</t>
+  </si>
+  <si>
+    <t>CALIDAD DE DATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Col M (idioma)</t>
+  </si>
+  <si>
+    <t>261/274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Col Y (tipoPersonalización)</t>
+  </si>
+  <si>
+    <t>203/274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Col Z (tamañoEmpresa)</t>
+  </si>
+  <si>
+    <t>108/274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Col N (adecuada)</t>
+  </si>
+  <si>
+    <t>28/274</t>
+  </si>
+  <si>
+    <t>Media: 20 días | Mediana: 3 días</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Tipo pers.</t>
+  </si>
+  <si>
+    <t>Tamaño</t>
+  </si>
+  <si>
+    <t>FACTOR: TIPO PERSONALIZACIÓN (col Y): tipo de personalización usada</t>
+  </si>
+  <si>
+    <t>FACTOR: TAMAÑO EMPRESA (col Z): tamaño estimado</t>
+  </si>
+  <si>
+    <t>FACTOR: GENÉRICO vs PERSONALIZADO REAL (basado en col Y)</t>
+  </si>
+  <si>
+    <t>Genérico (GN)</t>
+  </si>
+  <si>
+    <t>Personalizado real</t>
+  </si>
+  <si>
+    <t>CONCLUSIONES (generadas automáticamente a partir de los datos)</t>
+  </si>
+  <si>
+    <t>⚠ Col Z (tamañoEmpresa): solo 39.4% rellenada. Conclusiones sobre este factor NO son fiables.</t>
+  </si>
+  <si>
+    <t>⚠ Col N (adecuada): solo 10.2% rellenada. Conclusiones sobre este factor NO son fiables.</t>
+  </si>
+  <si>
+    <t>• EMAIL ÚNICO (col D): mejor resultado = no (4.2% Pos.Real) vs peor = sí (3.3%)</t>
+  </si>
+  <si>
+    <t>• PERSONALIZADO (col E): mejor resultado = sí (4.7% Pos.Real) vs peor = no (3.1%)</t>
+  </si>
+  <si>
+    <t>• IDIOMA (col M): mejor resultado = en (4.5% Pos.Real) vs peor = es (4.0%)</t>
+  </si>
+  <si>
+    <t>• ADECUACIÓN (col N): mejor resultado = ADECUADA (12.5% Pos.Real) vs peor = MUY ADECUADA (0.0%)</t>
+  </si>
+  <si>
+    <t>• REGIÓN: mejor resultado = Otro (3.8% Pos.Real) vs peor = Irlanda (0.0%)</t>
+  </si>
+  <si>
+    <t>• PERIODO TEMPORAL: mejor resultado = Antes ene-2026 (5.7% Pos.Real) vs peor = Desde 29-ene (+ recomendaciones) (1.8%)</t>
+  </si>
+  <si>
+    <t>• REMINDER (col B): mejor resultado = True (4.9% Pos.Real) vs peor = False (2.2%)</t>
+  </si>
+  <si>
+    <t>• TIPO PERSONALIZACIÓN (col Y): mejor resultado = JV (12.5% Pos.Real) vs peor = MLT (0.0%)</t>
+  </si>
+  <si>
+    <t>• TAMAÑO EMPRESA (col Z): mejor resultado = BT (15.9% Pos.Real) vs peor = GR (0.0%)</t>
+  </si>
+  <si>
+    <t>• GENÉRICO vs PERSONALIZADO REAL (basado en col Y): mejor resultado = Personalizado real (4.8% Pos.Real) vs peor = Genérico (GN) (3.5%)</t>
+  </si>
+  <si>
+    <t>NOTA: Las conclusiones anteriores son orientativas. Verificar que la muestra de cada factor es suficiente.</t>
   </si>
 </sst>
 </file>
@@ -64848,601 +64844,592 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1">
       <c r="A1" s="408" t="s">
-        <v>2008</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" customHeight="1">
       <c r="A2" t="s">
-        <v>2009</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="12.65" customHeight="1"/>
-    <row r="4" spans="1:2" ht="12.65" customHeight="1">
-      <c r="A4" s="408" t="s">
-        <v>2010</v>
-      </c>
-    </row>
+        <v>2059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="12.65" customHeight="1">
+      <c r="A3" t="s">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="12.65" customHeight="1"/>
     <row r="5" spans="1:2" ht="12.65" customHeight="1">
-      <c r="A5" t="s">
-        <v>2011</v>
+      <c r="A5" s="408" t="s">
+        <v>2008</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1">
       <c r="A6" t="s">
-        <v>2012</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="12.65" customHeight="1">
-      <c r="A7" s="408" t="s">
-        <v>2013</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="12.65" customHeight="1"/>
-    <row r="9" spans="1:2" ht="12.65" customHeight="1">
-      <c r="A9" s="408" t="s">
-        <v>2014</v>
-      </c>
-    </row>
+      <c r="A7" t="s">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="12.65" customHeight="1">
+      <c r="A8" s="408" t="s">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="12.65" customHeight="1"/>
     <row r="10" spans="1:2" ht="12.65" customHeight="1">
-      <c r="A10" t="s">
-        <v>2015</v>
-      </c>
-      <c r="B10" t="s">
-        <v>2016</v>
+      <c r="A10" s="408" t="s">
+        <v>2062</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="12.65" customHeight="1">
       <c r="A11" t="s">
-        <v>2017</v>
+        <v>2063</v>
       </c>
       <c r="B11" t="s">
-        <v>2018</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="12.65" customHeight="1">
       <c r="A12" t="s">
-        <v>2019</v>
+        <v>2064</v>
       </c>
       <c r="B12" t="s">
-        <v>2020</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="52" customHeight="1">
       <c r="A13" t="s">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="B13" t="s">
-        <v>765</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="12.65" customHeight="1">
       <c r="A14" t="s">
+        <v>2066</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2067</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="12.65" customHeight="1">
+      <c r="A15" t="s">
+        <v>2014</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="12.65" customHeight="1"/>
+    <row r="17" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A17" s="408" t="s">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="12.65" customHeight="1">
+      <c r="B18" t="s">
+        <v>2017</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="25" customHeight="1">
+      <c r="A19" t="s">
+        <v>2019</v>
+      </c>
+      <c r="B19">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A20" t="s">
+        <v>2020</v>
+      </c>
+      <c r="B20">
+        <v>81</v>
+      </c>
+      <c r="C20" s="406">
+        <v>0.29599999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="25" customHeight="1">
+      <c r="A21" t="s">
+        <v>2021</v>
+      </c>
+      <c r="B21">
+        <v>11</v>
+      </c>
+      <c r="C21" s="406">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A22" t="s">
         <v>2022</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B22">
+        <v>51</v>
+      </c>
+      <c r="C22" s="406">
+        <v>0.186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="25" customHeight="1">
+      <c r="A23" t="s">
         <v>2023</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="12.65" customHeight="1"/>
-    <row r="16" spans="1:2" ht="12.65" customHeight="1">
-      <c r="A16" s="408" t="s">
+      <c r="B23">
+        <v>14</v>
+      </c>
+      <c r="C23" s="406">
+        <v>5.0999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A24" t="s">
         <v>2024</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="12.65" customHeight="1">
-      <c r="B17" t="s">
+      <c r="B24">
+        <v>5</v>
+      </c>
+      <c r="C24" s="406">
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A25" t="s">
         <v>2025</v>
       </c>
-      <c r="C17" t="s">
+      <c r="B25">
+        <v>193</v>
+      </c>
+      <c r="C25" s="406">
+        <v>0.70399999999999996</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="12.65" customHeight="1"/>
+    <row r="27" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A27" s="408" t="s">
+        <v>2068</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A28" t="s">
+        <v>2069</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2070</v>
+      </c>
+      <c r="C28" s="406">
+        <v>0.95299999999999996</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A29" t="s">
+        <v>2071</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2072</v>
+      </c>
+      <c r="C29" s="406">
+        <v>0.74099999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A30" t="s">
+        <v>2073</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2074</v>
+      </c>
+      <c r="C30" s="406">
+        <v>0.39400000000000002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="12.65" customHeight="1">
+      <c r="A31" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2076</v>
+      </c>
+      <c r="C31" s="406">
+        <v>0.10199999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="12.65" customHeight="1"/>
+    <row r="33" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A33" s="408" t="s">
         <v>2026</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A18" t="s">
-        <v>2027</v>
-      </c>
-      <c r="B18">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="25" customHeight="1">
-      <c r="A19" t="s">
-        <v>2028</v>
-      </c>
-      <c r="B19">
-        <v>79</v>
-      </c>
-      <c r="C19" s="406">
-        <v>0.29199999999999998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A20" t="s">
-        <v>2029</v>
-      </c>
-      <c r="B20">
-        <v>11</v>
-      </c>
-      <c r="C20" s="406">
-        <v>4.1000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="25" customHeight="1">
-      <c r="A21" t="s">
-        <v>2030</v>
-      </c>
-      <c r="B21">
-        <v>50</v>
-      </c>
-      <c r="C21" s="406">
-        <v>0.185</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A22" t="s">
-        <v>2031</v>
-      </c>
-      <c r="B22">
-        <v>12</v>
-      </c>
-      <c r="C22" s="406">
-        <v>4.3999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="25" customHeight="1">
-      <c r="A23" t="s">
-        <v>2032</v>
-      </c>
-      <c r="B23">
-        <v>6</v>
-      </c>
-      <c r="C23" s="406">
-        <v>2.1999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A24" t="s">
-        <v>2033</v>
-      </c>
-      <c r="B24">
-        <v>192</v>
-      </c>
-      <c r="C24" s="406">
-        <v>0.70799999999999996</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="12.65" customHeight="1"/>
-    <row r="26" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A26" s="408" t="s">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A27" t="s">
-        <v>2035</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="12.65" customHeight="1"/>
-    <row r="29" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A29" s="408" t="s">
-        <v>2036</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A30" t="s">
-        <v>2037</v>
-      </c>
-      <c r="B30" t="s">
-        <v>2038</v>
-      </c>
-      <c r="C30" t="s">
-        <v>2039</v>
-      </c>
-      <c r="D30" t="s">
-        <v>2040</v>
-      </c>
-      <c r="E30" t="s">
-        <v>2041</v>
-      </c>
-      <c r="F30" t="s">
-        <v>2042</v>
-      </c>
-      <c r="G30" t="s">
-        <v>2043</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A31" t="s">
-        <v>138</v>
-      </c>
-      <c r="B31" t="s">
-        <v>2044</v>
-      </c>
-      <c r="D31" t="s">
-        <v>2045</v>
-      </c>
-      <c r="G31" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="12.65" customHeight="1">
-      <c r="A32" t="s">
-        <v>144</v>
-      </c>
-      <c r="B32" t="s">
-        <v>2044</v>
-      </c>
-      <c r="D32" t="s">
-        <v>2045</v>
-      </c>
-      <c r="F32" t="s">
-        <v>781</v>
-      </c>
-      <c r="G32" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="12.65" customHeight="1">
-      <c r="B33" t="s">
-        <v>2046</v>
-      </c>
-      <c r="C33" t="s">
-        <v>2045</v>
-      </c>
-      <c r="D33" t="s">
-        <v>2045</v>
-      </c>
-      <c r="G33" t="s">
-        <v>563</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="12.65" customHeight="1">
       <c r="A34" t="s">
-        <v>583</v>
-      </c>
-      <c r="B34" t="s">
-        <v>2046</v>
-      </c>
-      <c r="C34" t="s">
-        <v>1426</v>
-      </c>
-      <c r="D34" t="s">
-        <v>2045</v>
-      </c>
-      <c r="G34" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A35" t="s">
-        <v>626</v>
-      </c>
-      <c r="B35" s="407">
-        <v>45788</v>
-      </c>
-      <c r="C35" t="s">
-        <v>1426</v>
-      </c>
-      <c r="D35" t="s">
-        <v>2045</v>
-      </c>
-      <c r="F35" t="s">
-        <v>781</v>
-      </c>
-      <c r="G35" t="s">
-        <v>625</v>
-      </c>
-    </row>
+        <v>2077</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="12.65" customHeight="1"/>
     <row r="36" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A36" t="s">
-        <v>677</v>
-      </c>
-      <c r="B36" t="s">
-        <v>2047</v>
-      </c>
-      <c r="C36" t="s">
-        <v>1426</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1426</v>
-      </c>
-      <c r="E36" t="s">
-        <v>48</v>
-      </c>
-      <c r="G36" t="s">
-        <v>137</v>
+      <c r="A36" s="408" t="s">
+        <v>2027</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="12.65" customHeight="1">
       <c r="A37" t="s">
-        <v>928</v>
+        <v>2028</v>
       </c>
       <c r="B37" t="s">
-        <v>2048</v>
+        <v>2078</v>
       </c>
       <c r="C37" t="s">
-        <v>1426</v>
+        <v>2029</v>
       </c>
       <c r="D37" t="s">
-        <v>2045</v>
+        <v>2030</v>
       </c>
       <c r="E37" t="s">
-        <v>48</v>
+        <v>2031</v>
       </c>
       <c r="F37" t="s">
-        <v>781</v>
+        <v>2032</v>
       </c>
       <c r="G37" t="s">
-        <v>927</v>
+        <v>2079</v>
+      </c>
+      <c r="H37" t="s">
+        <v>2080</v>
+      </c>
+      <c r="I37" t="s">
+        <v>2033</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="12.65" customHeight="1">
       <c r="A38" t="s">
-        <v>1106</v>
+        <v>138</v>
       </c>
       <c r="B38" t="s">
-        <v>2048</v>
-      </c>
-      <c r="C38" t="s">
-        <v>2045</v>
+        <v>2034</v>
       </c>
       <c r="D38" t="s">
-        <v>2045</v>
+        <v>2035</v>
       </c>
       <c r="E38" t="s">
-        <v>48</v>
-      </c>
-      <c r="F38" t="s">
-        <v>2049</v>
+        <v>31</v>
       </c>
       <c r="G38" t="s">
-        <v>143</v>
+        <v>136</v>
+      </c>
+      <c r="H38" t="s">
+        <v>33</v>
+      </c>
+      <c r="I38" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="12.65" customHeight="1">
       <c r="A39" t="s">
-        <v>1111</v>
+        <v>144</v>
       </c>
       <c r="B39" t="s">
-        <v>2048</v>
-      </c>
-      <c r="C39" t="s">
-        <v>2045</v>
+        <v>2034</v>
       </c>
       <c r="D39" t="s">
-        <v>2045</v>
+        <v>1426</v>
       </c>
       <c r="E39" t="s">
         <v>48</v>
       </c>
       <c r="F39" t="s">
-        <v>2049</v>
+        <v>781</v>
       </c>
       <c r="G39" t="s">
+        <v>32</v>
+      </c>
+      <c r="H39" t="s">
+        <v>33</v>
+      </c>
+      <c r="I39" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A40" t="s">
-        <v>1528</v>
-      </c>
-      <c r="B40" s="407">
-        <v>46114</v>
+      <c r="B40" t="s">
+        <v>2036</v>
       </c>
       <c r="C40" t="s">
-        <v>1426</v>
+        <v>2035</v>
       </c>
       <c r="D40" t="s">
-        <v>2045</v>
-      </c>
-      <c r="F40" t="s">
-        <v>781</v>
+        <v>2035</v>
+      </c>
+      <c r="E40" t="s">
+        <v>31</v>
       </c>
       <c r="G40" t="s">
-        <v>137</v>
+        <v>387</v>
+      </c>
+      <c r="H40" t="s">
+        <v>33</v>
+      </c>
+      <c r="I40" t="s">
+        <v>563</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="12.65" customHeight="1">
       <c r="A41" t="s">
-        <v>1686</v>
-      </c>
-      <c r="B41" s="407">
-        <v>46144</v>
+        <v>583</v>
+      </c>
+      <c r="B41" t="s">
+        <v>2036</v>
       </c>
       <c r="C41" t="s">
         <v>1426</v>
       </c>
       <c r="D41" t="s">
-        <v>2045</v>
+        <v>2035</v>
       </c>
       <c r="E41" t="s">
         <v>48</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
+        <v>387</v>
+      </c>
+      <c r="H41" t="s">
+        <v>41</v>
+      </c>
+      <c r="I41" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A42" t="s">
+        <v>626</v>
+      </c>
+      <c r="B42" s="407">
+        <v>45788</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D42" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E42" t="s">
+        <v>31</v>
+      </c>
+      <c r="F42" t="s">
         <v>781</v>
       </c>
-      <c r="G41" t="s">
+      <c r="G42" t="s">
+        <v>387</v>
+      </c>
+      <c r="H42" t="s">
+        <v>33</v>
+      </c>
+      <c r="I42" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A43" t="s">
+        <v>677</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2037</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E43" t="s">
+        <v>48</v>
+      </c>
+      <c r="G43" t="s">
+        <v>32</v>
+      </c>
+      <c r="H43" t="s">
+        <v>33</v>
+      </c>
+      <c r="I43" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A44" t="s">
+        <v>928</v>
+      </c>
+      <c r="B44" t="s">
+        <v>2038</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D44" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E44" t="s">
+        <v>31</v>
+      </c>
+      <c r="F44" t="s">
+        <v>781</v>
+      </c>
+      <c r="G44" t="s">
+        <v>59</v>
+      </c>
+      <c r="H44" t="s">
+        <v>33</v>
+      </c>
+      <c r="I44" t="s">
         <v>927</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="12.65" customHeight="1"/>
-    <row r="43" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A43" s="408" t="s">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="12.65" customHeight="1">
-      <c r="B44" t="s">
-        <v>2051</v>
-      </c>
-      <c r="C44" t="s">
-        <v>2052</v>
-      </c>
-      <c r="D44" t="s">
-        <v>2053</v>
-      </c>
-      <c r="E44" t="s">
-        <v>2054</v>
-      </c>
-      <c r="F44" t="s">
-        <v>2055</v>
-      </c>
-      <c r="G44" t="s">
-        <v>2056</v>
-      </c>
-      <c r="H44" t="s">
-        <v>2057</v>
-      </c>
-      <c r="I44" t="s">
-        <v>2058</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="12.65" customHeight="1">
       <c r="A45" t="s">
-        <v>1426</v>
-      </c>
-      <c r="B45">
-        <v>6</v>
-      </c>
-      <c r="C45">
-        <v>19</v>
-      </c>
-      <c r="D45">
-        <v>8</v>
-      </c>
-      <c r="E45">
-        <v>2</v>
-      </c>
-      <c r="F45">
-        <v>108</v>
-      </c>
-      <c r="G45">
+        <v>1106</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2038</v>
+      </c>
+      <c r="C45" t="s">
+        <v>2035</v>
+      </c>
+      <c r="D45" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E45" t="s">
+        <v>48</v>
+      </c>
+      <c r="F45" t="s">
+        <v>2039</v>
+      </c>
+      <c r="G45" t="s">
+        <v>237</v>
+      </c>
+      <c r="H45" t="s">
+        <v>33</v>
+      </c>
+      <c r="I45" t="s">
         <v>143</v>
-      </c>
-      <c r="H45">
-        <v>17.5</v>
-      </c>
-      <c r="I45">
-        <v>4.2</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="12.65" customHeight="1">
       <c r="A46" t="s">
-        <v>2045</v>
-      </c>
-      <c r="B46">
-        <v>3</v>
-      </c>
-      <c r="C46">
-        <v>21</v>
-      </c>
-      <c r="D46">
-        <v>4</v>
-      </c>
-      <c r="E46">
-        <v>2</v>
-      </c>
-      <c r="F46">
-        <v>60</v>
-      </c>
-      <c r="G46">
-        <v>90</v>
-      </c>
-      <c r="H46">
-        <v>26.7</v>
-      </c>
-      <c r="I46">
-        <v>3.3</v>
+        <v>1111</v>
+      </c>
+      <c r="B46" t="s">
+        <v>2038</v>
+      </c>
+      <c r="C46" t="s">
+        <v>2035</v>
+      </c>
+      <c r="D46" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E46" t="s">
+        <v>48</v>
+      </c>
+      <c r="F46" t="s">
+        <v>2039</v>
+      </c>
+      <c r="G46" t="s">
+        <v>136</v>
+      </c>
+      <c r="H46" t="s">
+        <v>33</v>
+      </c>
+      <c r="I46" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="12.65" customHeight="1">
       <c r="A47" t="s">
-        <v>2056</v>
-      </c>
-      <c r="B47">
-        <v>9</v>
-      </c>
-      <c r="C47">
-        <v>40</v>
-      </c>
-      <c r="D47">
-        <v>12</v>
-      </c>
-      <c r="E47">
-        <v>4</v>
-      </c>
-      <c r="F47">
-        <v>168</v>
-      </c>
-      <c r="G47">
-        <v>233</v>
-      </c>
-      <c r="H47">
-        <v>21</v>
-      </c>
-      <c r="I47">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="12.65" customHeight="1"/>
-    <row r="49" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A49" s="408" t="s">
-        <v>2059</v>
-      </c>
-    </row>
+        <v>1528</v>
+      </c>
+      <c r="B47" s="407">
+        <v>46114</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D47" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F47" t="s">
+        <v>781</v>
+      </c>
+      <c r="H47" t="s">
+        <v>33</v>
+      </c>
+      <c r="I47" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A48" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B48" s="407">
+        <v>46144</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D48" t="s">
+        <v>2035</v>
+      </c>
+      <c r="E48" t="s">
+        <v>31</v>
+      </c>
+      <c r="F48" t="s">
+        <v>781</v>
+      </c>
+      <c r="H48" t="s">
+        <v>33</v>
+      </c>
+      <c r="I48" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="12.65" customHeight="1"/>
     <row r="50" spans="1:9" ht="12.65" customHeight="1">
-      <c r="B50" t="s">
-        <v>2051</v>
-      </c>
-      <c r="C50" t="s">
-        <v>2052</v>
-      </c>
-      <c r="D50" t="s">
-        <v>2053</v>
-      </c>
-      <c r="E50" t="s">
-        <v>2054</v>
-      </c>
-      <c r="F50" t="s">
-        <v>2055</v>
-      </c>
-      <c r="G50" t="s">
-        <v>2056</v>
-      </c>
-      <c r="H50" t="s">
-        <v>2057</v>
-      </c>
-      <c r="I50" t="s">
-        <v>2058</v>
+      <c r="A50" s="408" t="s">
+        <v>2040</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A51" t="s">
-        <v>2060</v>
-      </c>
-      <c r="B51">
-        <v>0</v>
-      </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51">
-        <v>0</v>
-      </c>
-      <c r="E51">
-        <v>0</v>
-      </c>
-      <c r="F51">
-        <v>16</v>
-      </c>
-      <c r="G51">
-        <v>18</v>
-      </c>
-      <c r="H51">
-        <v>11.1</v>
-      </c>
-      <c r="I51">
-        <v>0</v>
+      <c r="B51" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D51" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F51" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G51" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H51" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I51" t="s">
+        <v>2048</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="12.65" customHeight="1">
@@ -65450,425 +65437,425 @@
         <v>1426</v>
       </c>
       <c r="B52">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C52">
+        <v>19</v>
+      </c>
+      <c r="D52">
+        <v>8</v>
+      </c>
+      <c r="E52">
         <v>2</v>
       </c>
-      <c r="D52">
-        <v>3</v>
-      </c>
-      <c r="E52">
-        <v>0</v>
-      </c>
       <c r="F52">
-        <v>13</v>
+        <v>109</v>
       </c>
       <c r="G52">
-        <v>19</v>
+        <v>144</v>
       </c>
       <c r="H52">
-        <v>15.8</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="I52">
-        <v>5.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="12.65" customHeight="1">
       <c r="A53" t="s">
-        <v>2045</v>
+        <v>2035</v>
       </c>
       <c r="B53">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C53">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="D53">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E53">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F53">
-        <v>152</v>
+        <v>61</v>
       </c>
       <c r="G53">
-        <v>217</v>
+        <v>91</v>
       </c>
       <c r="H53">
-        <v>23.5</v>
+        <v>26.4</v>
       </c>
       <c r="I53">
-        <v>4.5999999999999996</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="12.65" customHeight="1">
       <c r="A54" t="s">
-        <v>2056</v>
+        <v>2046</v>
       </c>
       <c r="B54">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C54">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D54">
         <v>12</v>
       </c>
       <c r="E54">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F54">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="G54">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="H54">
-        <v>22</v>
+        <v>20.9</v>
       </c>
       <c r="I54">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="12.65" customHeight="1"/>
     <row r="56" spans="1:9" ht="12.65" customHeight="1">
       <c r="A56" s="408" t="s">
-        <v>2061</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="12.65" customHeight="1">
       <c r="B57" t="s">
-        <v>2051</v>
+        <v>2041</v>
       </c>
       <c r="C57" t="s">
-        <v>2052</v>
+        <v>2042</v>
       </c>
       <c r="D57" t="s">
-        <v>2053</v>
+        <v>2043</v>
       </c>
       <c r="E57" t="s">
-        <v>2054</v>
+        <v>2044</v>
       </c>
       <c r="F57" t="s">
-        <v>2055</v>
+        <v>2045</v>
       </c>
       <c r="G57" t="s">
-        <v>2056</v>
+        <v>2046</v>
       </c>
       <c r="H57" t="s">
-        <v>2057</v>
+        <v>2047</v>
       </c>
       <c r="I57" t="s">
-        <v>2058</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="12.65" customHeight="1">
       <c r="A58" t="s">
-        <v>48</v>
+        <v>1426</v>
       </c>
       <c r="B58">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C58">
         <v>8</v>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F58">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G58">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="H58">
-        <v>22.8</v>
+        <v>15.6</v>
       </c>
       <c r="I58">
-        <v>8.8000000000000007</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="12.65" customHeight="1">
       <c r="A59" t="s">
-        <v>31</v>
+        <v>2035</v>
       </c>
       <c r="B59">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C59">
+        <v>37</v>
+      </c>
+      <c r="D59">
+        <v>8</v>
+      </c>
+      <c r="E59">
         <v>4</v>
       </c>
-      <c r="D59">
-        <v>3</v>
-      </c>
-      <c r="E59">
-        <v>0</v>
-      </c>
       <c r="F59">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="G59">
-        <v>33</v>
+        <v>192</v>
       </c>
       <c r="H59">
-        <v>12.1</v>
+        <v>24</v>
       </c>
       <c r="I59">
-        <v>0</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="12.65" customHeight="1">
       <c r="A60" t="s">
-        <v>2056</v>
+        <v>2046</v>
       </c>
       <c r="B60">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C60">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="D60">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F60">
-        <v>67</v>
+        <v>183</v>
       </c>
       <c r="G60">
-        <v>90</v>
+        <v>256</v>
       </c>
       <c r="H60">
-        <v>18.899999999999999</v>
+        <v>21.9</v>
       </c>
       <c r="I60">
-        <v>5.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="12.65" customHeight="1"/>
     <row r="62" spans="1:9" ht="12.65" customHeight="1">
       <c r="A62" s="408" t="s">
-        <v>2062</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="12.65" customHeight="1">
       <c r="B63" t="s">
-        <v>2051</v>
+        <v>2041</v>
       </c>
       <c r="C63" t="s">
-        <v>2052</v>
+        <v>2042</v>
       </c>
       <c r="D63" t="s">
-        <v>2053</v>
+        <v>2043</v>
       </c>
       <c r="E63" t="s">
-        <v>2054</v>
+        <v>2044</v>
       </c>
       <c r="F63" t="s">
-        <v>2055</v>
+        <v>2045</v>
       </c>
       <c r="G63" t="s">
-        <v>2056</v>
+        <v>2046</v>
       </c>
       <c r="H63" t="s">
-        <v>2057</v>
+        <v>2047</v>
       </c>
       <c r="I63" t="s">
-        <v>2058</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="12.65" customHeight="1">
       <c r="A64" t="s">
-        <v>1752</v>
+        <v>48</v>
       </c>
       <c r="B64">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C64">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D64">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F64">
-        <v>5</v>
+        <v>79</v>
       </c>
       <c r="G64">
-        <v>7</v>
+        <v>111</v>
       </c>
       <c r="H64">
-        <v>28.6</v>
+        <v>21.6</v>
       </c>
       <c r="I64">
-        <v>14.3</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="12.65" customHeight="1">
       <c r="A65" t="s">
-        <v>1631</v>
+        <v>31</v>
       </c>
       <c r="B65">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C65">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="D65">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F65">
-        <v>9</v>
+        <v>103</v>
       </c>
       <c r="G65">
-        <v>9</v>
+        <v>150</v>
       </c>
       <c r="H65">
-        <v>0</v>
+        <v>24.7</v>
       </c>
       <c r="I65">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="12.65" customHeight="1">
       <c r="A66" t="s">
-        <v>1616</v>
+        <v>2046</v>
       </c>
       <c r="B66">
+        <v>11</v>
+      </c>
+      <c r="C66">
+        <v>50</v>
+      </c>
+      <c r="D66">
+        <v>13</v>
+      </c>
+      <c r="E66">
+        <v>5</v>
+      </c>
+      <c r="F66">
+        <v>182</v>
+      </c>
+      <c r="G66">
+        <v>261</v>
+      </c>
+      <c r="H66">
+        <v>23.4</v>
+      </c>
+      <c r="I66">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="68" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A68" s="408" t="s">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B69" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C69" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D69" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E69" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F69" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G69" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H69" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I69" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A70" t="s">
+        <v>1752</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70">
+        <v>1</v>
+      </c>
+      <c r="D70">
         <v>0</v>
       </c>
-      <c r="C66">
+      <c r="E70">
         <v>0</v>
       </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-      <c r="E66">
-        <v>0</v>
-      </c>
-      <c r="F66">
-        <v>9</v>
-      </c>
-      <c r="G66">
-        <v>9</v>
-      </c>
-      <c r="H66">
-        <v>0</v>
-      </c>
-      <c r="I66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A67" t="s">
-        <v>2056</v>
-      </c>
-      <c r="B67">
-        <v>1</v>
-      </c>
-      <c r="C67">
-        <v>1</v>
-      </c>
-      <c r="D67">
-        <v>0</v>
-      </c>
-      <c r="E67">
-        <v>0</v>
-      </c>
-      <c r="F67">
-        <v>23</v>
-      </c>
-      <c r="G67">
+      <c r="F70">
+        <v>6</v>
+      </c>
+      <c r="G70">
+        <v>8</v>
+      </c>
+      <c r="H70">
         <v>25</v>
       </c>
-      <c r="H67">
-        <v>8</v>
-      </c>
-      <c r="I67">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="12.65" customHeight="1"/>
-    <row r="69" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A69" s="408" t="s">
-        <v>2063</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" ht="12.65" customHeight="1">
-      <c r="B70" t="s">
-        <v>2051</v>
-      </c>
-      <c r="C70" t="s">
-        <v>2052</v>
-      </c>
-      <c r="D70" t="s">
-        <v>2053</v>
-      </c>
-      <c r="E70" t="s">
-        <v>2054</v>
-      </c>
-      <c r="F70" t="s">
-        <v>2055</v>
-      </c>
-      <c r="G70" t="s">
-        <v>2056</v>
-      </c>
-      <c r="H70" t="s">
-        <v>2057</v>
-      </c>
-      <c r="I70" t="s">
-        <v>2058</v>
+      <c r="I70">
+        <v>12.5</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="12.65" customHeight="1">
       <c r="A71" t="s">
-        <v>781</v>
+        <v>1631</v>
       </c>
       <c r="B71">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C71">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="D71">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E71">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F71">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="G71">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="H71">
-        <v>22.1</v>
+        <v>9.1</v>
       </c>
       <c r="I71">
-        <v>3.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="12.65" customHeight="1">
       <c r="A72" t="s">
-        <v>1105</v>
+        <v>1616</v>
       </c>
       <c r="B72">
         <v>0</v>
       </c>
       <c r="C72">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D72">
         <v>0</v>
@@ -65877,13 +65864,13 @@
         <v>0</v>
       </c>
       <c r="F72">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G72">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H72">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I72">
         <v>0</v>
@@ -65891,274 +65878,274 @@
     </row>
     <row r="73" spans="1:9" ht="12.65" customHeight="1">
       <c r="A73" t="s">
-        <v>2049</v>
+        <v>2046</v>
       </c>
       <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73">
         <v>2</v>
       </c>
-      <c r="C73">
+      <c r="D73">
+        <v>0</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>25</v>
+      </c>
+      <c r="G73">
+        <v>28</v>
+      </c>
+      <c r="H73">
+        <v>10.7</v>
+      </c>
+      <c r="I73">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="75" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A75" s="408" t="s">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B76" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C76" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D76" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E76" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F76" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G76" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H76" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I76" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A77" t="s">
+        <v>781</v>
+      </c>
+      <c r="B77">
+        <v>5</v>
+      </c>
+      <c r="C77">
+        <v>25</v>
+      </c>
+      <c r="D77">
         <v>6</v>
       </c>
-      <c r="D73">
-        <v>3</v>
-      </c>
-      <c r="E73">
+      <c r="E77">
+        <v>1</v>
+      </c>
+      <c r="F77">
+        <v>100</v>
+      </c>
+      <c r="G77">
+        <v>137</v>
+      </c>
+      <c r="H77">
+        <v>21.9</v>
+      </c>
+      <c r="I77">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A78" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B78">
+        <v>0</v>
+      </c>
+      <c r="C78">
         <v>2</v>
       </c>
-      <c r="F73">
-        <v>38</v>
-      </c>
-      <c r="G73">
-        <v>51</v>
-      </c>
-      <c r="H73">
-        <v>15.7</v>
-      </c>
-      <c r="I73">
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A74" t="s">
-        <v>1458</v>
-      </c>
-      <c r="B74">
+      <c r="D78">
         <v>0</v>
       </c>
-      <c r="C74">
-        <v>3</v>
-      </c>
-      <c r="D74">
+      <c r="E78">
         <v>0</v>
       </c>
-      <c r="E74">
+      <c r="F78">
+        <v>2</v>
+      </c>
+      <c r="G78">
+        <v>4</v>
+      </c>
+      <c r="H78">
+        <v>50</v>
+      </c>
+      <c r="I78">
         <v>0</v>
-      </c>
-      <c r="F74">
-        <v>10</v>
-      </c>
-      <c r="G74">
-        <v>13</v>
-      </c>
-      <c r="H74">
-        <v>23.1</v>
-      </c>
-      <c r="I74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A75" t="s">
-        <v>2056</v>
-      </c>
-      <c r="B75">
-        <v>7</v>
-      </c>
-      <c r="C75">
-        <v>36</v>
-      </c>
-      <c r="D75">
-        <v>9</v>
-      </c>
-      <c r="E75">
-        <v>3</v>
-      </c>
-      <c r="F75">
-        <v>149</v>
-      </c>
-      <c r="G75">
-        <v>204</v>
-      </c>
-      <c r="H75">
-        <v>21.1</v>
-      </c>
-      <c r="I75">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" ht="12.65" customHeight="1"/>
-    <row r="77" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A77" s="408" t="s">
-        <v>2064</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" ht="12.65" customHeight="1">
-      <c r="B78" t="s">
-        <v>2051</v>
-      </c>
-      <c r="C78" t="s">
-        <v>2052</v>
-      </c>
-      <c r="D78" t="s">
-        <v>2053</v>
-      </c>
-      <c r="E78" t="s">
-        <v>2054</v>
-      </c>
-      <c r="F78" t="s">
-        <v>2055</v>
-      </c>
-      <c r="G78" t="s">
-        <v>2056</v>
-      </c>
-      <c r="H78" t="s">
-        <v>2057</v>
-      </c>
-      <c r="I78" t="s">
-        <v>2058</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.65" customHeight="1">
       <c r="A79" t="s">
-        <v>2065</v>
+        <v>2039</v>
       </c>
       <c r="B79">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C79">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="D79">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E79">
         <v>2</v>
       </c>
       <c r="F79">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="G79">
-        <v>105</v>
+        <v>52</v>
       </c>
       <c r="H79">
-        <v>26.7</v>
+        <v>17.3</v>
       </c>
       <c r="I79">
-        <v>5.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="12.65" customHeight="1">
       <c r="A80" t="s">
-        <v>2066</v>
+        <v>1458</v>
       </c>
       <c r="B80">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C80">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D80">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E80">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F80">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="G80">
-        <v>108</v>
+        <v>13</v>
       </c>
       <c r="H80">
-        <v>20.399999999999999</v>
+        <v>23.1</v>
       </c>
       <c r="I80">
-        <v>1.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:9" ht="12.65" customHeight="1">
       <c r="A81" t="s">
-        <v>2067</v>
+        <v>2046</v>
       </c>
       <c r="B81">
+        <v>7</v>
+      </c>
+      <c r="C81">
+        <v>37</v>
+      </c>
+      <c r="D81">
+        <v>9</v>
+      </c>
+      <c r="E81">
         <v>3</v>
       </c>
-      <c r="C81">
+      <c r="F81">
+        <v>150</v>
+      </c>
+      <c r="G81">
+        <v>206</v>
+      </c>
+      <c r="H81">
+        <v>21.4</v>
+      </c>
+      <c r="I81">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="83" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A83" s="408" t="s">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B84" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C84" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D84" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E84" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F84" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G84" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H84" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I84" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A85" t="s">
+        <v>2054</v>
+      </c>
+      <c r="B85">
+        <v>6</v>
+      </c>
+      <c r="C85">
+        <v>22</v>
+      </c>
+      <c r="D85">
         <v>8</v>
       </c>
-      <c r="D81">
-        <v>2</v>
-      </c>
-      <c r="E81">
+      <c r="E85">
         <v>1</v>
       </c>
-      <c r="F81">
-        <v>44</v>
-      </c>
-      <c r="G81">
-        <v>58</v>
-      </c>
-      <c r="H81">
-        <v>19</v>
-      </c>
-      <c r="I81">
-        <v>5.2</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A82" t="s">
-        <v>2056</v>
-      </c>
-      <c r="B82">
-        <v>11</v>
-      </c>
-      <c r="C82">
-        <v>50</v>
-      </c>
-      <c r="D82">
-        <v>12</v>
-      </c>
-      <c r="E82">
-        <v>6</v>
-      </c>
-      <c r="F82">
-        <v>192</v>
-      </c>
-      <c r="G82">
-        <v>271</v>
-      </c>
-      <c r="H82">
-        <v>22.5</v>
-      </c>
-      <c r="I82">
-        <v>4.0999999999999996</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" ht="12.65" customHeight="1"/>
-    <row r="84" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A84" s="408" t="s">
-        <v>2068</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" ht="12.65" customHeight="1">
-      <c r="B85" t="s">
-        <v>2051</v>
-      </c>
-      <c r="C85" t="s">
-        <v>2052</v>
-      </c>
-      <c r="D85" t="s">
-        <v>2053</v>
-      </c>
-      <c r="E85" t="s">
-        <v>2054</v>
-      </c>
-      <c r="F85" t="s">
+      <c r="F85">
+        <v>68</v>
+      </c>
+      <c r="G85">
+        <v>105</v>
+      </c>
+      <c r="H85">
+        <v>26.7</v>
+      </c>
+      <c r="I85">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A86" t="s">
         <v>2055</v>
-      </c>
-      <c r="G85" t="s">
-        <v>2056</v>
-      </c>
-      <c r="H85" t="s">
-        <v>2057</v>
-      </c>
-      <c r="I85" t="s">
-        <v>2058</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A86" t="b">
-        <v>0</v>
       </c>
       <c r="B86">
         <v>2</v>
@@ -66170,257 +66157,861 @@
         <v>4</v>
       </c>
       <c r="E86">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F86">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="G86">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="H86">
-        <v>25.8</v>
+        <v>20.7</v>
       </c>
       <c r="I86">
-        <v>2.2000000000000002</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="87" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A87" t="b">
-        <v>1</v>
+      <c r="A87" t="s">
+        <v>2056</v>
       </c>
       <c r="B87">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C87">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D87">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E87">
         <v>1</v>
       </c>
       <c r="F87">
-        <v>135</v>
+        <v>44</v>
       </c>
       <c r="G87">
-        <v>182</v>
+        <v>58</v>
       </c>
       <c r="H87">
-        <v>20.9</v>
+        <v>19</v>
       </c>
       <c r="I87">
-        <v>4.9000000000000004</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="88" spans="1:9" ht="12.65" customHeight="1">
       <c r="A88" t="s">
-        <v>2056</v>
+        <v>2046</v>
       </c>
       <c r="B88">
         <v>11</v>
       </c>
       <c r="C88">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D88">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E88">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G88">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H88">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="I88">
-        <v>4.0999999999999996</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89" spans="1:9" ht="12.65" customHeight="1"/>
     <row r="90" spans="1:9" ht="12.65" customHeight="1">
       <c r="A90" s="408" t="s">
-        <v>2069</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" ht="12.65" customHeight="1"/>
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B91" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C91" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D91" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E91" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F91" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G91" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H91" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I91" t="s">
+        <v>2048</v>
+      </c>
+    </row>
     <row r="92" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A92" t="s">
-        <v>2070</v>
+      <c r="A92" t="b">
+        <v>0</v>
+      </c>
+      <c r="B92">
+        <v>2</v>
+      </c>
+      <c r="C92">
+        <v>22</v>
+      </c>
+      <c r="D92">
+        <v>5</v>
+      </c>
+      <c r="E92">
+        <v>4</v>
+      </c>
+      <c r="F92">
+        <v>58</v>
+      </c>
+      <c r="G92">
+        <v>91</v>
+      </c>
+      <c r="H92">
+        <v>26.4</v>
+      </c>
+      <c r="I92">
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="93" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A93" t="s">
-        <v>2071</v>
+      <c r="A93" t="b">
+        <v>1</v>
+      </c>
+      <c r="B93">
+        <v>9</v>
+      </c>
+      <c r="C93">
+        <v>29</v>
+      </c>
+      <c r="D93">
+        <v>9</v>
+      </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
+      <c r="F93">
+        <v>135</v>
+      </c>
+      <c r="G93">
+        <v>183</v>
+      </c>
+      <c r="H93">
+        <v>20.8</v>
+      </c>
+      <c r="I93">
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="94" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A94" s="408" t="s">
-        <v>2072</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A95" t="s">
-        <v>2073</v>
-      </c>
-    </row>
-    <row r="96" spans="1:9" ht="12.65" customHeight="1"/>
-    <row r="97" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A97" t="s">
-        <v>2074</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A94" t="s">
+        <v>2046</v>
+      </c>
+      <c r="B94">
+        <v>11</v>
+      </c>
+      <c r="C94">
+        <v>51</v>
+      </c>
+      <c r="D94">
+        <v>14</v>
+      </c>
+      <c r="E94">
+        <v>5</v>
+      </c>
+      <c r="F94">
+        <v>193</v>
+      </c>
+      <c r="G94">
+        <v>274</v>
+      </c>
+      <c r="H94">
+        <v>22.6</v>
+      </c>
+      <c r="I94">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="96" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A96" s="408" t="s">
+        <v>2081</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B97" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C97" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D97" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E97" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F97" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G97" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H97" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I97" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="12.65" customHeight="1">
       <c r="A98" t="s">
-        <v>2075</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" ht="12.65" customHeight="1">
+        <v>32</v>
+      </c>
+      <c r="B98">
+        <v>2</v>
+      </c>
+      <c r="C98">
+        <v>8</v>
+      </c>
+      <c r="D98">
+        <v>5</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+      <c r="F98">
+        <v>42</v>
+      </c>
+      <c r="G98">
+        <v>57</v>
+      </c>
+      <c r="H98">
+        <v>17.5</v>
+      </c>
+      <c r="I98">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="12.65" customHeight="1">
       <c r="A99" t="s">
-        <v>2076</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" ht="12.65" customHeight="1">
+        <v>237</v>
+      </c>
+      <c r="B99">
+        <v>1</v>
+      </c>
+      <c r="C99">
+        <v>4</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99">
+        <v>2</v>
+      </c>
+      <c r="F99">
+        <v>20</v>
+      </c>
+      <c r="G99">
+        <v>28</v>
+      </c>
+      <c r="H99">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="I99">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="12.65" customHeight="1">
       <c r="A100" t="s">
-        <v>2077</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="102" spans="1:1" ht="12.65" customHeight="1">
+        <v>59</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100">
+        <v>3</v>
+      </c>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="E100">
+        <v>0</v>
+      </c>
+      <c r="F100">
+        <v>4</v>
+      </c>
+      <c r="G100">
+        <v>8</v>
+      </c>
+      <c r="H100">
+        <v>50</v>
+      </c>
+      <c r="I100">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A101" t="s">
+        <v>174</v>
+      </c>
+      <c r="B101">
+        <v>0</v>
+      </c>
+      <c r="C101">
+        <v>0</v>
+      </c>
+      <c r="D101">
+        <v>0</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>2</v>
+      </c>
+      <c r="G101">
+        <v>2</v>
+      </c>
+      <c r="H101">
+        <v>0</v>
+      </c>
+      <c r="I101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="12.65" customHeight="1">
       <c r="A102" t="s">
-        <v>2078</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" ht="12.65" customHeight="1">
+        <v>136</v>
+      </c>
+      <c r="B102">
+        <v>2</v>
+      </c>
+      <c r="C102">
+        <v>13</v>
+      </c>
+      <c r="D102">
+        <v>3</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>44</v>
+      </c>
+      <c r="G102">
+        <v>62</v>
+      </c>
+      <c r="H102">
+        <v>24.2</v>
+      </c>
+      <c r="I102">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="12.65" customHeight="1">
       <c r="A103" t="s">
-        <v>2079</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="105" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A105" s="408" t="s">
-        <v>2080</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" ht="12.65" customHeight="1">
+        <v>1036</v>
+      </c>
+      <c r="B103">
+        <v>0</v>
+      </c>
+      <c r="C103">
+        <v>1</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>4</v>
+      </c>
+      <c r="G103">
+        <v>6</v>
+      </c>
+      <c r="H103">
+        <v>16.7</v>
+      </c>
+      <c r="I103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A104" t="s">
+        <v>160</v>
+      </c>
+      <c r="B104">
+        <v>0</v>
+      </c>
+      <c r="C104">
+        <v>5</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104">
+        <v>1</v>
+      </c>
+      <c r="F104">
+        <v>8</v>
+      </c>
+      <c r="G104">
+        <v>14</v>
+      </c>
+      <c r="H104">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="I104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A105" t="s">
+        <v>387</v>
+      </c>
+      <c r="B105">
+        <v>3</v>
+      </c>
+      <c r="C105">
+        <v>6</v>
+      </c>
+      <c r="D105">
+        <v>2</v>
+      </c>
+      <c r="E105">
+        <v>0</v>
+      </c>
+      <c r="F105">
+        <v>15</v>
+      </c>
+      <c r="G105">
+        <v>26</v>
+      </c>
+      <c r="H105">
+        <v>34.6</v>
+      </c>
+      <c r="I105">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="12.65" customHeight="1">
       <c r="A106" t="s">
-        <v>2081</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A107" t="s">
+        <v>2046</v>
+      </c>
+      <c r="B106">
+        <v>9</v>
+      </c>
+      <c r="C106">
+        <v>40</v>
+      </c>
+      <c r="D106">
+        <v>12</v>
+      </c>
+      <c r="E106">
+        <v>3</v>
+      </c>
+      <c r="F106">
+        <v>139</v>
+      </c>
+      <c r="G106">
+        <v>203</v>
+      </c>
+      <c r="H106">
+        <v>24.1</v>
+      </c>
+      <c r="I106">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="108" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A108" s="408" t="s">
         <v>2082</v>
       </c>
     </row>
-    <row r="108" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="109" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A109" t="s">
+    <row r="109" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B109" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C109" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D109" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E109" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F109" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G109" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H109" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I109" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A110" t="s">
+        <v>33</v>
+      </c>
+      <c r="B110">
+        <v>10</v>
+      </c>
+      <c r="C110">
+        <v>16</v>
+      </c>
+      <c r="D110">
+        <v>3</v>
+      </c>
+      <c r="E110">
+        <v>0</v>
+      </c>
+      <c r="F110">
+        <v>34</v>
+      </c>
+      <c r="G110">
+        <v>63</v>
+      </c>
+      <c r="H110">
+        <v>41.3</v>
+      </c>
+      <c r="I110">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A111" t="s">
+        <v>49</v>
+      </c>
+      <c r="B111">
+        <v>0</v>
+      </c>
+      <c r="C111">
+        <v>5</v>
+      </c>
+      <c r="D111">
+        <v>2</v>
+      </c>
+      <c r="E111">
+        <v>1</v>
+      </c>
+      <c r="F111">
+        <v>5</v>
+      </c>
+      <c r="G111">
+        <v>13</v>
+      </c>
+      <c r="H111">
+        <v>38.5</v>
+      </c>
+      <c r="I111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A112" t="s">
+        <v>112</v>
+      </c>
+      <c r="B112">
+        <v>0</v>
+      </c>
+      <c r="C112">
+        <v>4</v>
+      </c>
+      <c r="D112">
+        <v>1</v>
+      </c>
+      <c r="E112">
+        <v>0</v>
+      </c>
+      <c r="F112">
+        <v>5</v>
+      </c>
+      <c r="G112">
+        <v>10</v>
+      </c>
+      <c r="H112">
+        <v>40</v>
+      </c>
+      <c r="I112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A113" t="s">
+        <v>41</v>
+      </c>
+      <c r="B113">
+        <v>1</v>
+      </c>
+      <c r="C113">
+        <v>5</v>
+      </c>
+      <c r="D113">
+        <v>3</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>13</v>
+      </c>
+      <c r="G113">
+        <v>22</v>
+      </c>
+      <c r="H113">
+        <v>27.3</v>
+      </c>
+      <c r="I113">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A114" t="s">
+        <v>2046</v>
+      </c>
+      <c r="B114">
+        <v>11</v>
+      </c>
+      <c r="C114">
+        <v>30</v>
+      </c>
+      <c r="D114">
+        <v>9</v>
+      </c>
+      <c r="E114">
+        <v>1</v>
+      </c>
+      <c r="F114">
+        <v>57</v>
+      </c>
+      <c r="G114">
+        <v>108</v>
+      </c>
+      <c r="H114">
+        <v>38</v>
+      </c>
+      <c r="I114">
+        <v>10.199999999999999</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="116" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A116" s="408" t="s">
         <v>2083</v>
       </c>
     </row>
-    <row r="110" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A110" s="408" t="s">
+    <row r="117" spans="1:9" ht="12.65" customHeight="1">
+      <c r="B117" t="s">
+        <v>2041</v>
+      </c>
+      <c r="C117" t="s">
+        <v>2042</v>
+      </c>
+      <c r="D117" t="s">
+        <v>2043</v>
+      </c>
+      <c r="E117" t="s">
+        <v>2044</v>
+      </c>
+      <c r="F117" t="s">
+        <v>2045</v>
+      </c>
+      <c r="G117" t="s">
+        <v>2046</v>
+      </c>
+      <c r="H117" t="s">
+        <v>2047</v>
+      </c>
+      <c r="I117" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A118" t="s">
         <v>2084</v>
       </c>
-    </row>
-    <row r="111" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="112" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A112" t="s">
+      <c r="B118">
+        <v>2</v>
+      </c>
+      <c r="C118">
+        <v>8</v>
+      </c>
+      <c r="D118">
+        <v>5</v>
+      </c>
+      <c r="E118">
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>42</v>
+      </c>
+      <c r="G118">
+        <v>57</v>
+      </c>
+      <c r="H118">
+        <v>17.5</v>
+      </c>
+      <c r="I118">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A119" t="s">
         <v>2085</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A113" t="s">
+      <c r="B119">
+        <v>7</v>
+      </c>
+      <c r="C119">
+        <v>32</v>
+      </c>
+      <c r="D119">
+        <v>7</v>
+      </c>
+      <c r="E119">
+        <v>3</v>
+      </c>
+      <c r="F119">
+        <v>97</v>
+      </c>
+      <c r="G119">
+        <v>146</v>
+      </c>
+      <c r="H119">
+        <v>26.7</v>
+      </c>
+      <c r="I119">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A120" t="s">
+        <v>2046</v>
+      </c>
+      <c r="B120">
+        <v>9</v>
+      </c>
+      <c r="C120">
+        <v>40</v>
+      </c>
+      <c r="D120">
+        <v>12</v>
+      </c>
+      <c r="E120">
+        <v>3</v>
+      </c>
+      <c r="F120">
+        <v>139</v>
+      </c>
+      <c r="G120">
+        <v>203</v>
+      </c>
+      <c r="H120">
+        <v>24.1</v>
+      </c>
+      <c r="I120">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="122" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A122" s="408" t="s">
         <v>2086</v>
       </c>
     </row>
-    <row r="114" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A114" t="s">
+    <row r="123" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="124" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A124" s="408" t="s">
         <v>2087</v>
       </c>
     </row>
-    <row r="115" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A115" s="408" t="s">
+    <row r="125" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A125" s="408" t="s">
         <v>2088</v>
       </c>
     </row>
-    <row r="116" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A116" t="s">
+    <row r="126" spans="1:9" ht="12.65" customHeight="1"/>
+    <row r="127" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A127" t="s">
         <v>2089</v>
       </c>
     </row>
-    <row r="117" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="118" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A118" t="s">
+    <row r="128" spans="1:9" ht="12.65" customHeight="1">
+      <c r="A128" t="s">
         <v>2090</v>
       </c>
     </row>
-    <row r="119" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A119" t="s">
+    <row r="129" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A129" t="s">
         <v>2091</v>
       </c>
     </row>
-    <row r="120" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="121" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A121" t="s">
+    <row r="130" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A130" t="s">
         <v>2092</v>
       </c>
     </row>
-    <row r="122" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A122" s="408" t="s">
+    <row r="131" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A131" t="s">
         <v>2093</v>
       </c>
     </row>
-    <row r="123" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A123" t="s">
+    <row r="132" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A132" t="s">
         <v>2094</v>
       </c>
     </row>
-    <row r="124" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A124" t="s">
+    <row r="133" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A133" t="s">
         <v>2095</v>
       </c>
     </row>
-    <row r="125" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="126" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A126" t="s">
+    <row r="134" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A134" t="s">
         <v>2096</v>
       </c>
     </row>
-    <row r="127" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A127" t="s">
+    <row r="135" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A135" t="s">
         <v>2097</v>
       </c>
     </row>
-    <row r="128" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A128" t="s">
+    <row r="136" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A136" t="s">
         <v>2098</v>
       </c>
     </row>
-    <row r="129" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A129" s="408" t="s">
+    <row r="137" spans="1:1" ht="12.65" customHeight="1"/>
+    <row r="138" spans="1:1" ht="12.65" customHeight="1">
+      <c r="A138" s="408" t="s">
         <v>2099</v>
       </c>
     </row>
-    <row r="130" spans="1:1" ht="12.65" customHeight="1">
-      <c r="A130" s="408" t="s">
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="131" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="132" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="133" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="134" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="135" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="136" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="137" spans="1:1" ht="12.65" customHeight="1"/>
-    <row r="138" spans="1:1" ht="12.65" customHeight="1"/>
     <row r="139" spans="1:1" ht="12.65" customHeight="1"/>
     <row r="140" spans="1:1" ht="12.65" customHeight="1"/>
     <row r="141" spans="1:1" ht="12.65" customHeight="1"/>

</xml_diff>

<commit_message>
Actualizar Excel clientes (j-clientes-gle.xlsx)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88153b17ae7a9f01/documentos/TRABAJOS AUTONOMOS/JURADA/j-busqueda clientes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1398" documentId="13_ncr:1_{DF388099-A258-48E4-8A4C-6C022E777824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57F3A1CB-0EF8-42A6-BA25-0394A92EFD2F}"/>
+  <xr:revisionPtr revIDLastSave="1416" documentId="13_ncr:1_{DF388099-A258-48E4-8A4C-6C022E777824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DF9117F-7C92-49CB-84D9-AA2BCC5880B1}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="0">clientes!$A$1:$Y$58</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3784" uniqueCount="2156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3794" uniqueCount="2160">
   <si>
     <t>fechaEmail</t>
   </si>
@@ -6555,6 +6555,18 @@
   </si>
   <si>
     <t>Web 403. Traductores inglés/árabe/francés, colaboradores países árabes. Versión francesa del sitio. Clientela principal árabe/francófona. Inglés secundario, sin evidencia clientes UK/US.</t>
+  </si>
+  <si>
+    <t>info@perezdevargas.es / marbella@perezdevargas.com / estepona@perezdevargas.com</t>
+  </si>
+  <si>
+    <t>FBERNAL Abogados</t>
+  </si>
+  <si>
+    <t>Pedro Fernández</t>
+  </si>
+  <si>
+    <t>pedrofernandez@abogaciaextranjeria.es</t>
   </si>
 </sst>
 </file>
@@ -26801,12 +26813,18 @@
       <c r="AG313" s="84"/>
     </row>
     <row r="314" spans="1:33" ht="11.5" customHeight="1">
-      <c r="A314" s="414"/>
+      <c r="A314" s="412">
+        <v>46077</v>
+      </c>
       <c r="B314" s="289"/>
       <c r="C314" s="289"/>
       <c r="D314" s="86"/>
-      <c r="E314" s="87"/>
-      <c r="F314" s="87"/>
+      <c r="E314" s="87" t="s">
+        <v>26</v>
+      </c>
+      <c r="F314" s="87" t="s">
+        <v>55</v>
+      </c>
       <c r="G314" s="87"/>
       <c r="H314" s="201" t="s">
         <v>2096</v>
@@ -27025,12 +27043,18 @@
       <c r="AG318" s="97"/>
     </row>
     <row r="319" spans="1:33" ht="11.5" customHeight="1">
-      <c r="A319" s="412"/>
+      <c r="A319" s="412">
+        <v>46077</v>
+      </c>
       <c r="B319" s="288"/>
       <c r="C319" s="288"/>
       <c r="D319" s="81"/>
-      <c r="E319" s="82"/>
-      <c r="F319" s="82"/>
+      <c r="E319" s="82" t="s">
+        <v>26</v>
+      </c>
+      <c r="F319" s="82" t="s">
+        <v>55</v>
+      </c>
       <c r="G319" s="82"/>
       <c r="H319" s="199" t="s">
         <v>2109</v>
@@ -27127,6 +27151,9 @@
         <v>2114</v>
       </c>
       <c r="J321" s="201"/>
+      <c r="K321" s="200" t="s">
+        <v>2156</v>
+      </c>
       <c r="L321" s="201" t="s">
         <v>2120</v>
       </c>
@@ -27157,19 +27184,33 @@
       <c r="AG321" s="87"/>
     </row>
     <row r="322" spans="1:33" ht="11.5" customHeight="1">
-      <c r="A322" s="425"/>
+      <c r="A322" s="412">
+        <v>46077</v>
+      </c>
       <c r="B322" s="290"/>
       <c r="C322" s="290"/>
       <c r="D322" s="88"/>
       <c r="E322" s="89"/>
       <c r="F322" s="89"/>
       <c r="G322" s="89"/>
-      <c r="H322" s="198"/>
-      <c r="J322" s="198"/>
+      <c r="H322" s="198" t="s">
+        <v>2157</v>
+      </c>
+      <c r="I322" s="200" t="s">
+        <v>1729</v>
+      </c>
+      <c r="J322" s="198" t="s">
+        <v>2158</v>
+      </c>
+      <c r="K322" s="200" t="s">
+        <v>2159</v>
+      </c>
       <c r="L322" s="198"/>
       <c r="M322" s="256"/>
       <c r="N322" s="89"/>
-      <c r="O322" s="89"/>
+      <c r="O322" s="89" t="s">
+        <v>1703</v>
+      </c>
       <c r="P322" s="89"/>
       <c r="Q322" s="89"/>
       <c r="R322" s="89"/>

</xml_diff>

<commit_message>
Actualizar Excel clientes, presupuestos y carpeta en_curso
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88153b17ae7a9f01/documentos/TRABAJOS AUTONOMOS/JURADA/j-busqueda clientes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_A7EF37BD59B216A1919E58397C9D2DAA6E9EA21E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9538D6FD-5157-4423-957F-0B85042B97DC}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{0AFA8464-F26A-41CE-9FAC-2E395A515B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4925D569-AD13-4800-8678-F6DA847A4DA4}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5267" uniqueCount="3070">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5269" uniqueCount="3070">
   <si>
     <t>fechaEmail</t>
   </si>
@@ -9310,7 +9310,7 @@
     <numFmt numFmtId="167" formatCode="d\-m\-yy;@"/>
     <numFmt numFmtId="168" formatCode="d\-m\-yyyy"/>
   </numFmts>
-  <fonts count="57">
+  <fonts count="58">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -9662,6 +9662,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="26">
     <fill>
@@ -9906,7 +9913,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="454">
+  <cellXfs count="456">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -11209,6 +11216,12 @@
     <xf numFmtId="0" fontId="55" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="57" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -11225,10 +11238,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20239,7 +20248,7 @@
       <c r="F149" s="104" t="s">
         <v>58</v>
       </c>
-      <c r="G149" s="113" t="s">
+      <c r="G149" s="455" t="s">
         <v>97</v>
       </c>
       <c r="H149" s="143" t="s">
@@ -20443,14 +20452,18 @@
       <c r="C153" s="365" t="s">
         <v>776</v>
       </c>
-      <c r="D153" s="108"/>
+      <c r="D153" s="108">
+        <v>46086</v>
+      </c>
       <c r="E153" s="81" t="s">
         <v>27</v>
       </c>
       <c r="F153" s="81" t="s">
         <v>58</v>
       </c>
-      <c r="G153" s="81"/>
+      <c r="G153" s="416" t="s">
+        <v>97</v>
+      </c>
       <c r="H153" s="142" t="s">
         <v>913</v>
       </c>
@@ -31718,14 +31731,18 @@
       </c>
       <c r="B344" s="204"/>
       <c r="C344" s="380"/>
-      <c r="D344" s="86"/>
+      <c r="D344" s="86">
+        <v>46080</v>
+      </c>
       <c r="E344" s="88" t="s">
         <v>27</v>
       </c>
       <c r="F344" s="88" t="s">
         <v>58</v>
       </c>
-      <c r="G344" s="88"/>
+      <c r="G344" s="403" t="s">
+        <v>27</v>
+      </c>
       <c r="H344" s="122" t="s">
         <v>2095</v>
       </c>
@@ -32491,7 +32508,7 @@
         <v>1780</v>
       </c>
       <c r="P354" s="420"/>
-      <c r="Q354" s="420" t="s">
+      <c r="Q354" s="402" t="s">
         <v>2228</v>
       </c>
       <c r="R354" s="420"/>
@@ -32749,7 +32766,7 @@
       <c r="J358" s="119" t="s">
         <v>2300</v>
       </c>
-      <c r="K358" s="120" t="s">
+      <c r="K358" s="454" t="s">
         <v>2301</v>
       </c>
       <c r="L358" s="119" t="s">

</xml_diff>

<commit_message>
Actualizar Excel de clientes
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rocio\OneDrive\documentos\TRABAJOS AUTONOMOS\JURADA\j-busqueda clientes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A2029E-8E0C-4E20-9F58-3C284BA7BF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0691193-CE52-40CA-AC12-5DD3C742F909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1260" yWindow="-120" windowWidth="27660" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5266" uniqueCount="3069">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5268" uniqueCount="3071">
   <si>
     <t>fechaEmail</t>
   </si>
@@ -9294,6 +9294,12 @@
   </si>
   <si>
     <t>1-1n</t>
+  </si>
+  <si>
+    <t>tarifas ofrecidas</t>
+  </si>
+  <si>
+    <t>0,11/ pal / 30-40 por doc</t>
   </si>
 </sst>
 </file>
@@ -9910,7 +9916,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="456">
+  <cellXfs count="457">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -11219,6 +11225,9 @@
     <xf numFmtId="0" fontId="55" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="25" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -11546,7 +11555,9 @@
       <c r="AA1" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="26"/>
+      <c r="AB1" s="415" t="s">
+        <v>3069</v>
+      </c>
       <c r="AC1" s="26"/>
       <c r="AD1" s="26"/>
       <c r="AE1" s="26"/>
@@ -27266,7 +27277,9 @@
       <c r="AA270" s="360" t="s">
         <v>34</v>
       </c>
-      <c r="AB270" s="360"/>
+      <c r="AB270" s="456" t="s">
+        <v>3070</v>
+      </c>
       <c r="AC270" s="360"/>
       <c r="AD270" s="360"/>
       <c r="AE270" s="360"/>

</xml_diff>

<commit_message>
Actualizar Excel de clientes jurada
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rocio\OneDrive\documentos\TRABAJOS AUTONOMOS\JURADA\j-busqueda clientes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0691193-CE52-40CA-AC12-5DD3C742F909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F773AF29-691D-415A-A88F-79748947A016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1260" yWindow="-120" windowWidth="27660" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5268" uniqueCount="3071">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5269" uniqueCount="3071">
   <si>
     <t>fechaEmail</t>
   </si>
@@ -18320,14 +18320,18 @@
         <v>45987</v>
       </c>
       <c r="C115" s="365"/>
-      <c r="D115" s="109"/>
+      <c r="D115" s="109">
+        <v>46114</v>
+      </c>
       <c r="E115" s="102" t="s">
         <v>27</v>
       </c>
       <c r="F115" s="102" t="s">
         <v>27</v>
       </c>
-      <c r="G115" s="102"/>
+      <c r="G115" s="85" t="s">
+        <v>939</v>
+      </c>
       <c r="H115" s="124" t="s">
         <v>726</v>
       </c>

</xml_diff>

<commit_message>
clientes-gle: actualización del Excel de clientes
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rocio\OneDrive\documentos\TRABAJOS AUTONOMOS\JURADA\j-busqueda clientes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2A7A41-F0CC-436A-BECA-FEBB3DDE851D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA96B70-6F6B-4B2F-8DBC-688FBCA75807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1260" yWindow="-120" windowWidth="27660" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5270" uniqueCount="3072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5270" uniqueCount="3073">
   <si>
     <t>fechaEmail</t>
   </si>
@@ -9303,6 +9303,9 @@
   </si>
   <si>
     <t>v / 0,9/pal (rebajo desde 11 céntimos)</t>
+  </si>
+  <si>
+    <t>v / 0,11/pal /30-40 doc</t>
   </si>
 </sst>
 </file>
@@ -22752,7 +22755,7 @@
         <v>46076.958333333343</v>
       </c>
       <c r="C192" s="399" t="s">
-        <v>1112</v>
+        <v>3072</v>
       </c>
       <c r="D192" s="109">
         <v>46036</v>

</xml_diff>

<commit_message>
Actualiza Excel de clientes leads jurada
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88153b17ae7a9f01/documentos/TRABAJOS AUTONOMOS/JURADA/j-busqueda clientes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_D63F57C2E7E2542D700A1305F6CE983A5695B77D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{195BA87F-D777-4390-AE5B-F85746C539A4}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_D63F57C2E7E2542D700A1305F6CE983A5695B77D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33FB9B58-734D-4C8F-B6D2-4D421C711F1B}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5638" uniqueCount="3350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5639" uniqueCount="3350">
   <si>
     <t>para día</t>
   </si>
@@ -21571,7 +21571,9 @@
       <c r="F154" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="G154" s="101"/>
+      <c r="G154" s="406" t="s">
+        <v>154</v>
+      </c>
       <c r="H154" s="146" t="s">
         <v>934</v>
       </c>

</xml_diff>

<commit_message>
Actualizar Excel de clientes (j-clientes-gle.xlsx)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88153b17ae7a9f01/documentos/TRABAJOS AUTONOMOS/JURADA/j-busqueda clientes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_8D71D4E3FF54086EB3E5708B7890922AE0578CDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AC1CC79-5B46-4F19-A930-9ED8F7B01944}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_8D71D4E3FF54086EB3E5708B7890922AE0578CDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CB0FE34-902F-45A7-9FF3-4862903B6F36}"/>
   <bookViews>
-    <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clientes" sheetId="1" r:id="rId1"/>
@@ -10993,7 +10993,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="495">
+  <cellXfs count="497">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -12405,6 +12405,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="67" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -12421,6 +12423,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -73742,19 +73748,19 @@
   <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="1" max="1" width="11" style="496" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="32" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" customWidth="1"/>
     <col min="6" max="6" width="42" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="70" customWidth="1"/>
+    <col min="9" max="9" width="50.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="13">
-      <c r="A1" s="492" t="s">
+      <c r="A1" s="495" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="492" t="s">
@@ -73783,7 +73789,9 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="37.5">
-      <c r="A2" s="493"/>
+      <c r="A2" s="496">
+        <v>46238</v>
+      </c>
       <c r="B2" t="s">
         <v>3365</v>
       </c>
@@ -73802,7 +73810,6 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="37.5">
-      <c r="A3" s="493"/>
       <c r="B3" t="s">
         <v>3370</v>
       </c>
@@ -73824,7 +73831,6 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="25">
-      <c r="A4" s="493"/>
       <c r="B4" t="s">
         <v>3375</v>
       </c>
@@ -73846,7 +73852,6 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="25">
-      <c r="A5" s="493"/>
       <c r="B5" t="s">
         <v>3380</v>
       </c>
@@ -73865,7 +73870,6 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="25">
-      <c r="A6" s="493"/>
       <c r="B6" t="s">
         <v>3385</v>
       </c>
@@ -73884,7 +73888,6 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="25">
-      <c r="A7" s="493"/>
       <c r="B7" t="s">
         <v>3390</v>
       </c>
@@ -73903,7 +73906,6 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="25">
-      <c r="A8" s="493"/>
       <c r="B8" t="s">
         <v>3394</v>
       </c>
@@ -73922,7 +73924,6 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="25">
-      <c r="A9" s="493"/>
       <c r="B9" t="s">
         <v>3398</v>
       </c>
@@ -73944,7 +73945,6 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="25">
-      <c r="A10" s="493"/>
       <c r="B10" t="s">
         <v>3402</v>
       </c>
@@ -73961,6 +73961,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Actualizar Excel de busqueda de clientes
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/j-busqueda clientes/j-clientes-gle.xlsx
+++ b/j-busqueda clientes/j-clientes-gle.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88153b17ae7a9f01/documentos/TRABAJOS AUTONOMOS/JURADA/j-busqueda clientes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_8D71D4E3FF54086EB3E5708B7890922AE0578CDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00EA212E-46F1-42D4-A663-893CCCCD5380}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_8D71D4E3FF54086EB3E5708B7890922AE0578CDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58D0681B-671C-4933-8668-5C1F50641B05}"/>
   <bookViews>
     <workbookView xWindow="810" yWindow="-110" windowWidth="24900" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10993,7 +10993,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="497">
+  <cellXfs count="498">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -12407,6 +12407,9 @@
     </xf>
     <xf numFmtId="166" fontId="67" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -22717,8 +22720,8 @@
         <v>46035</v>
       </c>
       <c r="C171" s="379"/>
-      <c r="D171" s="76" t="s">
-        <v>1014</v>
+      <c r="D171" s="497">
+        <v>46259</v>
       </c>
       <c r="E171" s="76" t="s">
         <v>64</v>
@@ -22726,7 +22729,9 @@
       <c r="F171" s="76" t="s">
         <v>64</v>
       </c>
-      <c r="G171" s="76"/>
+      <c r="G171" s="450" t="s">
+        <v>149</v>
+      </c>
       <c r="H171" s="116" t="s">
         <v>1015</v>
       </c>

</xml_diff>